<commit_message>
Checklist: coluna Fonte de medição ao lado de Como medir (planilha Google e script)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5swnHARNHJ12oc84LP2b9
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Glossário" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist variáveis'!$A$4:$Q$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist variáveis'!$A$4:$R$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Glossário'!$A$4:$D$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -756,26 +756,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -788,7 +789,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Proposta de 02/10/2026 (Pedro + Claude), atualizada em 03/10/2026 com o documento da equipe (Hellis); não validada pelo grupo. I3, V5 e V6 são novas e ainda sem definição nem escala. Nota 5 = mais crítico. Faixa fixa = valor absoluto (provisória: calibrar com os dados reais). Quintil = nota relativa entre os 21 pontos (Quintil 1 = 20% com menor valor). Preencha as colunas amarelas (N, O e P): Sim / Não / Parcial / Pendente. 'Fonte confirmada' = a base existe e é acessível; 'Dado existe na fonte' = a variável está lá, na escala do círculo de 300 m, e cobre os 21 pontos. Termos explicados na aba Glossário.</t>
+          <t>Proposta de 02/10/2026 (Pedro + Claude), atualizada em 03/10/2026 com o documento da equipe (Hellis); não validada pelo grupo. I3, V5 e V6 são novas e ainda sem definição nem escala. Nota 5 = mais crítico. Faixa fixa = valor absoluto (provisória: calibrar com os dados reais). Quintil = nota relativa entre os 21 pontos (Quintil 1 = 20% com menor valor). Preencha as colunas amarelas (O, P e Q): Sim / Não / Parcial / Pendente. 'Fonte confirmada' = a base existe e é acessível; 'Dado existe na fonte' = a variável está lá, na escala do círculo de 300 m, e cobre os 21 pontos. Termos explicados na aba Glossário.</t>
         </is>
       </c>
     </row>
@@ -815,65 +816,70 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>Fonte de medição</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>Tipo de nota</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Nota 1</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Nota 2</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Nota 3</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Nota 4</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Nota 5</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Origem da faixa</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Recomendação</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Fonte</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Fonte confirmada?</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Dado existe na fonte?</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Busca prévia (Claude)</t>
         </is>
@@ -900,67 +906,68 @@
           <t>Média de eventos por ano nas 3 últimas estações chuvosas</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Faixa fixa</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>&lt; 1</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>1–2</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>3–4</t>
         </is>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="J5" s="11" t="inlineStr">
         <is>
           <t>5–6</t>
         </is>
       </c>
-      <c r="J5" s="12" t="inlineStr">
+      <c r="K5" s="12" t="inlineStr">
         <is>
           <t>≥ 7</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>Planilha original (provisória)</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>Manter — peso alto</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>Ficha preenchida com a EMLURB (agora); ocorrências do COP e da Defesa Civil (confirmação)</t>
         </is>
       </c>
-      <c r="N5" s="13" t="inlineStr">
+      <c r="O5" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O5" s="13" t="inlineStr">
+      <c r="P5" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P5" s="14" t="inlineStr">
+      <c r="Q5" s="14" t="inlineStr">
         <is>
           <t>Pedido ao COP via tutora/CGM. 156 só para conferir. Calibrar faixas com a distribuição real. 'Recorrência histórica' (documento da equipe) fica aqui se for o mesmo que frequência (pendência 16).</t>
         </is>
       </c>
-      <c r="Q5" s="6" t="inlineStr">
+      <c r="R5" s="6" t="inlineStr">
         <is>
           <t>Não verificado: depende de pedido aos órgãos.</t>
         </is>
@@ -987,67 +994,68 @@
           <t>Altura máxima da água e tempo para baixar; nota = média das duas notas, arredondada para cima</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Faixa fixa</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Altura &lt; 10 cm / baixa em &lt; 1 h</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>10–30 cm (tornozelo) / 1–3 h</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="I6" s="10" t="inlineStr">
         <is>
           <t>30–50 cm (joelho) / 3–6 h</t>
         </is>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>50–100 cm (cintura) / 6–12 h</t>
         </is>
       </c>
-      <c r="J6" s="12" t="inlineStr">
+      <c r="K6" s="12" t="inlineStr">
         <is>
           <t>&gt; 100 cm / &gt; 12 h</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>Planilha original (provisória); regra da média: proposta Claude</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>Manter — peso alto</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>Ficha EMLURB; escuta com Defesa Civil e moradores</t>
         </is>
       </c>
-      <c r="N6" s="13" t="inlineStr">
+      <c r="O6" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O6" s="13" t="inlineStr">
+      <c r="P6" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P6" s="14" t="inlineStr">
+      <c r="Q6" s="14" t="inlineStr">
         <is>
           <t>Extensão da mancha fica registrada como informação, sem nota própria.</t>
         </is>
       </c>
-      <c r="Q6" s="6" t="inlineStr">
+      <c r="R6" s="6" t="inlineStr">
         <is>
           <t>Não verificado: dado de campo.</t>
         </is>
@@ -1074,67 +1082,68 @@
           <t>O escoamento trava com a maré alta?</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Classe</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Não influencia</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="I7" s="10" t="inlineStr">
         <is>
           <t>Agrava ocasionalmente</t>
         </is>
       </c>
-      <c r="I7" s="11" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J7" s="12" t="inlineStr">
+      <c r="K7" s="12" t="inlineStr">
         <is>
           <t>Alaga dependendo da maré / escoamento bloqueado</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>Planilha original</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Ficha EMLURB; APAC; tábua de marés</t>
         </is>
       </c>
-      <c r="N7" s="13" t="inlineStr">
+      <c r="O7" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O7" s="13" t="inlineStr">
+      <c r="P7" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P7" s="14" t="inlineStr">
+      <c r="Q7" s="14" t="inlineStr">
         <is>
           <t>Notas 2 e 4 ficam para casos intermediários, se a EMLURB indicar.</t>
         </is>
       </c>
-      <c r="Q7" s="6" t="inlineStr">
+      <c r="R7" s="6" t="inlineStr">
         <is>
           <t>APAC confirmada na busca; tábua de marés não verificada.</t>
         </is>
@@ -1161,67 +1170,68 @@
           <t>Distância do ponto ao curso d'água mais próximo (m); quanto mais perto, maior a nota</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Quintil (invertido)</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>Quintil mais distante</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>Quintil 2</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>Quintil 3</t>
         </is>
       </c>
-      <c r="I8" s="11" t="inlineStr">
+      <c r="J8" s="11" t="inlineStr">
         <is>
           <t>Quintil 4</t>
         </is>
       </c>
-      <c r="J8" s="12" t="inlineStr">
+      <c r="K8" s="12" t="inlineStr">
         <is>
           <t>Quintil mais próximo</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>Regra de quintis da planilha original</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="M8" s="6" t="inlineStr">
         <is>
           <t>Manter — peso menor (suscetibilidade)</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>Shapefile próprio da rede hidrográfica; ESIG – recursos hídricos</t>
         </is>
       </c>
-      <c r="N8" s="13" t="inlineStr">
+      <c r="O8" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O8" s="13" t="inlineStr">
+      <c r="P8" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P8" s="14" t="inlineStr">
+      <c r="Q8" s="14" t="inlineStr">
         <is>
           <t>Reprojetar para EPSG:31985. Conferir se os canais estão no arquivo.</t>
         </is>
       </c>
-      <c r="Q8" s="6" t="inlineStr">
+      <c r="R8" s="6" t="inlineStr">
         <is>
           <t>ESIG com recursos hídricos confirmado na busca (não aberto).</t>
         </is>
@@ -1248,67 +1258,68 @@
           <t>% do círculo de 300 m com vegetação ou solo permeável; quanto menos verde, maior a nota</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Faixa fixa</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>&gt; 40%</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>30–40%</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>20–30%</t>
         </is>
       </c>
-      <c r="I9" s="11" t="inlineStr">
+      <c r="J9" s="11" t="inlineStr">
         <is>
           <t>10–20%</t>
         </is>
       </c>
-      <c r="J9" s="12" t="inlineStr">
+      <c r="K9" s="12" t="inlineStr">
         <is>
           <t>&lt; 10%</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>Planilha original (provisória)</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
         <is>
           <t>Manter — peso menor (suscetibilidade)</t>
         </is>
       </c>
-      <c r="M9" s="6" t="inlineStr">
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>MapBiomas (30 m); alternativa: edificações do ESIG</t>
         </is>
       </c>
-      <c r="N9" s="13" t="inlineStr">
+      <c r="O9" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O9" s="13" t="inlineStr">
+      <c r="P9" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P9" s="14" t="inlineStr">
+      <c r="Q9" s="14" t="inlineStr">
         <is>
           <t>Se quase todos os pontos ficarem em &lt; 10%, trocar por quintis.</t>
         </is>
       </c>
-      <c r="Q9" s="6" t="inlineStr">
+      <c r="R9" s="6" t="inlineStr">
         <is>
           <t>Não verificado.</t>
         </is>
@@ -1335,67 +1346,68 @@
           <t>Cota do ponto menos a cota média do círculo (m); quanto mais baixo, maior a nota</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Quintil (invertido)</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>Quintil mais alto</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>Quintil 2</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>Quintil 3</t>
         </is>
       </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>Quintil 4</t>
         </is>
       </c>
-      <c r="J10" s="12" t="inlineStr">
+      <c r="K10" s="12" t="inlineStr">
         <is>
           <t>Quintil mais baixo</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>Proposta Claude (quintis)</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="M10" s="6" t="inlineStr">
         <is>
           <t>Condicional — só com curvas de nível ou modelo de terreno</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr">
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>Condepe/Fidem — Acervo Cartográfico (curvas de nível); ESIG (a verificar)</t>
         </is>
       </c>
-      <c r="N10" s="13" t="inlineStr">
+      <c r="O10" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O10" s="13" t="inlineStr">
+      <c r="P10" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P10" s="14" t="inlineStr">
+      <c r="Q10" s="14" t="inlineStr">
         <is>
           <t>Medida mais objetiva de acúmulo de água. 'Relevo' do documento da equipe.</t>
         </is>
       </c>
-      <c r="Q10" s="6" t="inlineStr">
+      <c r="R10" s="6" t="inlineStr">
         <is>
           <t>Condepe/Fidem localizado na busca: curvas de 1 m na área urbana (não aberto).</t>
         </is>
@@ -1422,67 +1434,68 @@
           <t>Moradores no círculo de 300 m (soma de população × fração da célula dentro do círculo)</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Quintil</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Quintil 1 (20% menores)</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Quintil 2</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="I11" s="10" t="inlineStr">
         <is>
           <t>Quintil 3</t>
         </is>
       </c>
-      <c r="I11" s="11" t="inlineStr">
+      <c r="J11" s="11" t="inlineStr">
         <is>
           <t>Quintil 4</t>
         </is>
       </c>
-      <c r="J11" s="12" t="inlineStr">
+      <c r="K11" s="12" t="inlineStr">
         <is>
           <t>Quintil 5 (20% maiores)</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>Planilha original</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M11" s="6" t="inlineStr">
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>IBGE — Grade Estatística 2022 (células de 200 × 200 m)</t>
         </is>
       </c>
-      <c r="N11" s="13" t="inlineStr">
+      <c r="O11" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O11" s="13" t="inlineStr">
+      <c r="P11" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P11" s="14" t="inlineStr">
+      <c r="Q11" s="14" t="inlineStr">
         <is>
           <t>No painel, mostrar também o valor em 1 km.</t>
         </is>
       </c>
-      <c r="Q11" s="6" t="inlineStr">
+      <c r="R11" s="6" t="inlineStr">
         <is>
           <t>Confirmado na busca (não baixado).</t>
         </is>
@@ -1509,67 +1522,68 @@
           <t>Nº de escolas, creches e unidades de saúde no círculo</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Faixa fixa</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
         <is>
           <t>Nenhum</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="I12" s="10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I12" s="11" t="inlineStr">
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>3–4</t>
         </is>
       </c>
-      <c r="J12" s="12" t="inlineStr">
+      <c r="K12" s="12" t="inlineStr">
         <is>
           <t>≥ 5 ou hospital/UPA no círculo</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>Proposta Claude (provisória)</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="M12" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M12" s="6" t="inlineStr">
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>Portal de dados abertos (escolas municipais, UBS, hospitais, rede de saúde); IBGE — CNEFE 2022 (ensino e saúde); CNES/DATASUS</t>
         </is>
       </c>
-      <c r="N12" s="13" t="inlineStr">
+      <c r="O12" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O12" s="13" t="inlineStr">
+      <c r="P12" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P12" s="14" t="inlineStr">
+      <c r="Q12" s="14" t="inlineStr">
         <is>
           <t>Inclui 'hospitais/escolas atingidos' do documento da equipe (sem contar duas vezes no Impacto). Perguntar se 'equipamentos públicos' inclui outros (CRAS, abrigos). Calibrar com as contagens reais.</t>
         </is>
       </c>
-      <c r="Q12" s="6" t="inlineStr">
+      <c r="R12" s="6" t="inlineStr">
         <is>
           <t>CNEFE confirmado na busca (não baixado). Bases do portal localizadas em 03/10 (não abertas).</t>
         </is>
@@ -1596,67 +1610,68 @@
           <t>Nº de comércios e serviços no círculo</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Quintil</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Quintil 1 (20% menores)</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Quintil 2</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>Quintil 3</t>
         </is>
       </c>
-      <c r="I13" s="11" t="inlineStr">
+      <c r="J13" s="11" t="inlineStr">
         <is>
           <t>Quintil 4</t>
         </is>
       </c>
-      <c r="J13" s="12" t="inlineStr">
+      <c r="K13" s="12" t="inlineStr">
         <is>
           <t>Quintil 5 (20% maiores)</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>Planilha original</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M13" s="6" t="inlineStr">
+      <c r="N13" s="6" t="inlineStr">
         <is>
           <t>IBGE — CNEFE 2022 (outras finalidades); IPTU (tipo de empreendimento)</t>
         </is>
       </c>
-      <c r="N13" s="13" t="inlineStr">
+      <c r="O13" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O13" s="13" t="inlineStr">
+      <c r="P13" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P13" s="14" t="inlineStr">
+      <c r="Q13" s="14" t="inlineStr">
         <is>
           <t>'Outras finalidades' pode incluir templos e órgãos públicos. Inclui 'perdas econômicas' do documento da equipe, que não tem fonte própria.</t>
         </is>
       </c>
-      <c r="Q13" s="6" t="inlineStr">
+      <c r="R13" s="6" t="inlineStr">
         <is>
           <t>CNEFE confirmado na busca (não baixado).</t>
         </is>
@@ -1683,63 +1698,64 @@
           <t>% de moradores com 60+ anos ou 0–4 anos nos setores do círculo (ponderado pela área)</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Quintil</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>Quintil 1 (20% menores)</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Quintil 2</t>
         </is>
       </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>Quintil 3</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr">
+      <c r="J14" s="11" t="inlineStr">
         <is>
           <t>Quintil 4</t>
         </is>
       </c>
-      <c r="J14" s="12" t="inlineStr">
+      <c r="K14" s="12" t="inlineStr">
         <is>
           <t>Quintil 5 (20% maiores)</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>Planilha original</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="M14" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr">
+      <c r="N14" s="6" t="inlineStr">
         <is>
           <t>IBGE — Agregados por setor 2022 (idade)</t>
         </is>
       </c>
-      <c r="N14" s="13" t="inlineStr">
+      <c r="O14" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O14" s="13" t="inlineStr">
+      <c r="P14" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P14" s="14" t="inlineStr"/>
-      <c r="Q14" s="6" t="inlineStr">
+      <c r="Q14" s="14" t="inlineStr"/>
+      <c r="R14" s="6" t="inlineStr">
         <is>
           <t>Idade por setor confirmada na busca (não baixado).</t>
         </is>
@@ -1766,67 +1782,68 @@
           <t>% da área do círculo em favelas e comunidades urbanas (IBGE 2022) ou em ZEIS 1</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Faixa fixa</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>&lt; 10%</t>
         </is>
       </c>
-      <c r="H15" s="10" t="inlineStr">
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>10–25%</t>
         </is>
       </c>
-      <c r="I15" s="11" t="inlineStr">
+      <c r="J15" s="11" t="inlineStr">
         <is>
           <t>25–50%</t>
         </is>
       </c>
-      <c r="J15" s="12" t="inlineStr">
+      <c r="K15" s="12" t="inlineStr">
         <is>
           <t>&gt; 50%</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>Proposta Claude (provisória)</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>Manter — substitui o V1 se a malha 2022 existir</t>
         </is>
       </c>
-      <c r="M15" s="6" t="inlineStr">
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>IBGE — Favelas e Comunidades Urbanas 2022 (malha); ZEIS do Plano Diretor e relação de favelas (portal)</t>
         </is>
       </c>
-      <c r="N15" s="13" t="inlineStr">
+      <c r="O15" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O15" s="13" t="inlineStr">
+      <c r="P15" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P15" s="14" t="inlineStr">
+      <c r="Q15" s="14" t="inlineStr">
         <is>
           <t>Mais atual que o IVS (2010). ZEIS 2 (terrenos vazios) não conta.</t>
         </is>
       </c>
-      <c r="Q15" s="6" t="inlineStr">
+      <c r="R15" s="6" t="inlineStr">
         <is>
           <t>ZEIS e relação de favelas localizadas no portal (não abertas); malha IBGE não verificada.</t>
         </is>
@@ -1853,67 +1870,68 @@
           <t>% de domicílios do tipo casa nos setores do círculo</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>Quintil</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>Quintil 1 (20% menores)</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>Quintil 2</t>
         </is>
       </c>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="I16" s="10" t="inlineStr">
         <is>
           <t>Quintil 3</t>
         </is>
       </c>
-      <c r="I16" s="11" t="inlineStr">
+      <c r="J16" s="11" t="inlineStr">
         <is>
           <t>Quintil 4</t>
         </is>
       </c>
-      <c r="J16" s="12" t="inlineStr">
+      <c r="K16" s="12" t="inlineStr">
         <is>
           <t>Quintil 5 (20% maiores)</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>Proposta Claude (quintis)</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M16" s="6" t="inlineStr">
+      <c r="N16" s="6" t="inlineStr">
         <is>
           <t>IBGE — Agregados por setor 2022 (tipo de domicílio)</t>
         </is>
       </c>
-      <c r="N16" s="13" t="inlineStr">
+      <c r="O16" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O16" s="13" t="inlineStr">
+      <c r="P16" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P16" s="14" t="inlineStr">
+      <c r="Q16" s="14" t="inlineStr">
         <is>
           <t>Casa térrea é mais atingida que apartamento.</t>
         </is>
       </c>
-      <c r="Q16" s="6" t="inlineStr">
+      <c r="R16" s="6" t="inlineStr">
         <is>
           <t>Não verificado se a variável está no arquivo por setor.</t>
         </is>
@@ -1940,39 +1958,40 @@
           <t>Definição pendente (pendência 15)</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr"/>
-      <c r="G17" s="9" t="inlineStr"/>
-      <c r="H17" s="10" t="inlineStr"/>
-      <c r="I17" s="11" t="inlineStr"/>
-      <c r="J17" s="12" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr"/>
+      <c r="H17" s="9" t="inlineStr"/>
+      <c r="I17" s="10" t="inlineStr"/>
+      <c r="J17" s="11" t="inlineStr"/>
+      <c r="K17" s="12" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>Documento da equipe (Hellis, 03/10/2026)</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr">
         <is>
           <t>Nova — só entra com definição e fonte</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="13" t="inlineStr">
+      <c r="N17" s="6" t="inlineStr"/>
+      <c r="O17" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O17" s="13" t="inlineStr">
+      <c r="P17" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P17" s="14" t="inlineStr">
+      <c r="Q17" s="14" t="inlineStr">
         <is>
           <t>Pedir a definição a Hellis antes de procurar dado.</t>
         </is>
       </c>
-      <c r="Q17" s="6" t="inlineStr">
+      <c r="R17" s="6" t="inlineStr">
         <is>
           <t>Não pesquisado.</t>
         </is>
@@ -1999,39 +2018,40 @@
           <t>Definição pendente (pendência 15)</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr"/>
-      <c r="F18" s="8" t="inlineStr"/>
-      <c r="G18" s="9" t="inlineStr"/>
-      <c r="H18" s="10" t="inlineStr"/>
-      <c r="I18" s="11" t="inlineStr"/>
-      <c r="J18" s="12" t="inlineStr"/>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr"/>
+      <c r="H18" s="9" t="inlineStr"/>
+      <c r="I18" s="10" t="inlineStr"/>
+      <c r="J18" s="11" t="inlineStr"/>
+      <c r="K18" s="12" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>Documento da equipe (Hellis, 03/10/2026)</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="M18" s="6" t="inlineStr">
         <is>
           <t>Nova — só entra com definição e fonte</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr"/>
-      <c r="N18" s="13" t="inlineStr">
+      <c r="N18" s="6" t="inlineStr"/>
+      <c r="O18" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O18" s="13" t="inlineStr">
+      <c r="P18" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P18" s="14" t="inlineStr">
+      <c r="Q18" s="14" t="inlineStr">
         <is>
           <t>Pode absorver o V4 (tipo de moradia) e o I2 (esgoto). Pedir a definição a Hellis.</t>
         </is>
       </c>
-      <c r="Q18" s="6" t="inlineStr">
+      <c r="R18" s="6" t="inlineStr">
         <is>
           <t>Não pesquisado.</t>
         </is>
@@ -2058,67 +2078,68 @@
           <t>Maior IVS entre as UDHs que tocam o círculo</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>Faixa fixa</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>Muito baixa (0–0,200)</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>Baixa (0,201–0,300)</t>
         </is>
       </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>Média (0,301–0,400)</t>
         </is>
       </c>
-      <c r="I19" s="11" t="inlineStr">
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>Alta (0,401–0,500)</t>
         </is>
       </c>
-      <c r="J19" s="12" t="inlineStr">
+      <c r="K19" s="12" t="inlineStr">
         <is>
           <t>Muito alta (&gt; 0,500)</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="L19" s="6" t="inlineStr">
         <is>
           <t>Faixas do Ipea (conferir no Atlas)</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
         <is>
           <t>Plano B — só se o V3 não estiver disponível</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="N19" s="6" t="inlineStr">
         <is>
           <t>Ipea — Atlas da Vulnerabilidade Social (UDH)</t>
         </is>
       </c>
-      <c r="N19" s="13" t="inlineStr">
+      <c r="O19" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O19" s="13" t="inlineStr">
+      <c r="P19" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P19" s="14" t="inlineStr">
+      <c r="Q19" s="14" t="inlineStr">
         <is>
           <t>Base do Censo 2010.</t>
         </is>
       </c>
-      <c r="Q19" s="6" t="inlineStr">
+      <c r="R19" s="6" t="inlineStr">
         <is>
           <t>Site confirmado na busca; faixas e ano-base a confirmar.</t>
         </is>
@@ -2145,67 +2166,68 @@
           <t>Classe da via mais importante afetada pelo alagamento (no trecho: a própria via)</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Classe</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>Ruas</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>Demais avenidas</t>
         </is>
       </c>
-      <c r="H20" s="10" t="inlineStr">
+      <c r="I20" s="10" t="inlineStr">
         <is>
           <t>Corredor de transporte urbano secundário</t>
         </is>
       </c>
-      <c r="I20" s="11" t="inlineStr">
+      <c r="J20" s="11" t="inlineStr">
         <is>
           <t>Corredor de transporte urbano principal</t>
         </is>
       </c>
-      <c r="J20" s="12" t="inlineStr">
+      <c r="K20" s="12" t="inlineStr">
         <is>
           <t>Corredor de transporte metropolitano</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>Pedro (03/10/2026)</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M20" s="6" t="inlineStr">
+      <c r="N20" s="6" t="inlineStr">
         <is>
           <t>Corredores de ônibus (portal de dados abertos); hierarquia viária e corredores (CTTU / Grande Recife)</t>
         </is>
       </c>
-      <c r="N20" s="13" t="inlineStr">
+      <c r="O20" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O20" s="13" t="inlineStr">
+      <c r="P20" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P20" s="14" t="inlineStr">
+      <c r="Q20" s="14" t="inlineStr">
         <is>
           <t>Interdição registrada pela CTTU serve só para conferir a nota (não soma). Junta 'vias principais' e 'interrupção do trânsito' do documento da equipe. Confirmar qual base classifica os corredores em metropolitano / urbano principal / urbano secundário (pendência 17).</t>
         </is>
       </c>
-      <c r="Q20" s="6" t="inlineStr">
+      <c r="R20" s="6" t="inlineStr">
         <is>
           <t>Corredores de ônibus localizados no portal (não abertos); classificação dos corredores não verificada.</t>
         </is>
@@ -2232,67 +2254,68 @@
           <t>% de domicílios sem ligação à rede de esgoto nos setores do círculo</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr"/>
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Quintil</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>Quintil 1 (20% menores)</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>Quintil 2</t>
         </is>
       </c>
-      <c r="H21" s="10" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Quintil 3</t>
         </is>
       </c>
-      <c r="I21" s="11" t="inlineStr">
+      <c r="J21" s="11" t="inlineStr">
         <is>
           <t>Quintil 4</t>
         </is>
       </c>
-      <c r="J21" s="12" t="inlineStr">
+      <c r="K21" s="12" t="inlineStr">
         <is>
           <t>Quintil 5 (20% maiores)</t>
         </is>
       </c>
-      <c r="K21" s="6" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>Proposta Claude (quintis)</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr">
+      <c r="M21" s="6" t="inlineStr">
         <is>
           <t>Manter</t>
         </is>
       </c>
-      <c r="M21" s="6" t="inlineStr">
+      <c r="N21" s="6" t="inlineStr">
         <is>
           <t>IBGE — Agregados por setor 2022 (esgotamento); Compesa</t>
         </is>
       </c>
-      <c r="N21" s="13" t="inlineStr">
+      <c r="O21" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O21" s="13" t="inlineStr">
+      <c r="P21" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P21" s="14" t="inlineStr">
+      <c r="Q21" s="14" t="inlineStr">
         <is>
           <t>Quintis porque a cobertura de esgoto no Recife é baixa e faixas fixas podem saturar. Pode passar para o V6 (infraestrutura precária).</t>
         </is>
       </c>
-      <c r="Q21" s="6" t="inlineStr">
+      <c r="R21" s="6" t="inlineStr">
         <is>
           <t>Esgotamento por setor confirmado na busca (não baixado).</t>
         </is>
@@ -2319,39 +2342,40 @@
           <t>Definição pendente (pendência 15)</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr"/>
-      <c r="G22" s="9" t="inlineStr"/>
-      <c r="H22" s="10" t="inlineStr"/>
-      <c r="I22" s="11" t="inlineStr"/>
-      <c r="J22" s="12" t="inlineStr"/>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="7" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr"/>
+      <c r="H22" s="9" t="inlineStr"/>
+      <c r="I22" s="10" t="inlineStr"/>
+      <c r="J22" s="11" t="inlineStr"/>
+      <c r="K22" s="12" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>Documento da equipe (Hellis, 03/10/2026)</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr">
+      <c r="M22" s="6" t="inlineStr">
         <is>
           <t>Nova — só entra com definição e fonte</t>
         </is>
       </c>
-      <c r="M22" s="6" t="inlineStr"/>
-      <c r="N22" s="13" t="inlineStr">
+      <c r="N22" s="6" t="inlineStr"/>
+      <c r="O22" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O22" s="13" t="inlineStr">
+      <c r="P22" s="13" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="P22" s="14" t="inlineStr">
+      <c r="Q22" s="14" t="inlineStr">
         <is>
           <t>Leitura possível: comunidade sem rota alternativa quando o ponto alaga (malha viária). Confirmar com Hellis.</t>
         </is>
       </c>
-      <c r="Q22" s="6" t="inlineStr">
+      <c r="R22" s="6" t="inlineStr">
         <is>
           <t>Não pesquisado.</t>
         </is>
@@ -2363,94 +2387,94 @@
           <t>Resumo</t>
         </is>
       </c>
-      <c r="N24" s="21" t="inlineStr">
+      <c r="O24" s="21" t="inlineStr">
         <is>
           <t>Fonte confirmada</t>
         </is>
       </c>
-      <c r="O24" s="21" t="inlineStr">
+      <c r="P24" s="21" t="inlineStr">
         <is>
           <t>Dado existe</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="M25" s="22" t="inlineStr">
+      <c r="N25" s="22" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="N25" s="23">
-        <f>COUNTIF(N$5:N$22,$M25)</f>
-        <v/>
-      </c>
       <c r="O25" s="23">
-        <f>COUNTIF(O$5:O$22,$M25)</f>
+        <f>COUNTIF(O$5:O$22,$N25)</f>
+        <v/>
+      </c>
+      <c r="P25" s="23">
+        <f>COUNTIF(P$5:P$22,$N25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="M26" s="22" t="inlineStr">
+      <c r="N26" s="22" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
-      <c r="N26" s="23">
-        <f>COUNTIF(N$5:N$22,$M26)</f>
-        <v/>
-      </c>
       <c r="O26" s="23">
-        <f>COUNTIF(O$5:O$22,$M26)</f>
+        <f>COUNTIF(O$5:O$22,$N26)</f>
+        <v/>
+      </c>
+      <c r="P26" s="23">
+        <f>COUNTIF(P$5:P$22,$N26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="M27" s="22" t="inlineStr">
+      <c r="N27" s="22" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N27" s="23">
-        <f>COUNTIF(N$5:N$22,$M27)</f>
-        <v/>
-      </c>
       <c r="O27" s="23">
-        <f>COUNTIF(O$5:O$22,$M27)</f>
+        <f>COUNTIF(O$5:O$22,$N27)</f>
+        <v/>
+      </c>
+      <c r="P27" s="23">
+        <f>COUNTIF(P$5:P$22,$N27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="M28" s="22" t="inlineStr">
+      <c r="N28" s="22" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="N28" s="23">
-        <f>COUNTIF(N$5:N$22,$M28)</f>
-        <v/>
-      </c>
       <c r="O28" s="23">
-        <f>COUNTIF(O$5:O$22,$M28)</f>
+        <f>COUNTIF(O$5:O$22,$N28)</f>
+        <v/>
+      </c>
+      <c r="P28" s="23">
+        <f>COUNTIF(P$5:P$22,$N28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="M29" s="24" t="inlineStr">
+      <c r="N29" s="24" t="inlineStr">
         <is>
           <t>Variáveis com fonte e dado confirmados</t>
         </is>
       </c>
-      <c r="O29" s="25">
-        <f>COUNTIFS(N5:N22,"Sim",O5:O22,"Sim")&amp;" de "&amp;ROWS(N5:N22)</f>
+      <c r="P29" s="25">
+        <f>COUNTIFS(O5:O22,"Sim",P5:P22,"Sim")&amp;" de "&amp;ROWS(O5:O22)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q22"/>
+  <autoFilter ref="A4:R22"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A2:R2"/>
   </mergeCells>
-  <conditionalFormatting sqref="N5:O22">
+  <conditionalFormatting sqref="O5:P22">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Sim"</formula>
     </cfRule>
@@ -2462,7 +2486,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="N5:O22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O5:P22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não,Parcial,Pendente"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
I1: como medir pela hierarquia viária da CTTU (planilha, script e documento-chave)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5swnHARNHJ12oc84LP2b9
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
@@ -2163,7 +2163,10 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Classe da via mais importante afetada pelo alagamento (no trecho: a própria via)</t>
+          <t>Passo 1 — Identificar a via afetada. Trecho (Linha ou Vários): a própria via do trecho. Ponto num cruzamento: todas as vias que se cruzam ali; vale a mais importante. Ponto isolado numa via: a própria via.
+Passo 2 — Classificar a via estritamente pela hierarquia viária da CTTU (cttu.recife.pe.gov.br/sistema-viario e Classificação Hierárquica): corredor de transporte metropolitano, corredor de transporte urbano principal, corredor de transporte urbano secundário ou via fora dos corredores. O nome da via (avenida ou rua) não conta.
+Passo 3 — Converter a classe em nota pela escala das colunas G a K.
+Regras: se a classe muda ao longo da via, vale a classe no trecho do ponto; se o ponto pega mais de uma via, vale a de nota mais alta; interdição registrada pela CTTU só confere a nota, não soma.</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
I4 Proximidade a infraestrutura crítica (faixas de Pedro); I1 com fonte confirmada por Pedro; pendência 18
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5swnHARNHJ12oc84LP2b9
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Glossário" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist variáveis'!$A$4:$R$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist variáveis'!$A$4:$R$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Glossário'!$A$4:$D$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -756,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2169,7 +2169,11 @@
 Regras: se a classe muda ao longo da via, vale a classe no trecho do ponto; se o ponto pega mais de uma via, vale a de nota mais alta; interdição registrada pela CTTU só confere a nota, não soma.</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Sistema viário | CTTU</t>
+        </is>
+      </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Classe</t>
@@ -2217,12 +2221,12 @@
       </c>
       <c r="O20" s="13" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="P20" s="13" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="Q20" s="14" t="inlineStr">
@@ -2384,100 +2388,188 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Impacto</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Proximidade a infraestrutura crítica</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Distância em linha reta (EPSG:31985) do ponto, ou da linha do trecho, até a infraestrutura crítica mais próxima. Infraestrutura crítica = estrutura cuja interrupção por alagamento deixa sem serviço essencial uma área maior que o entorno do ponto: estação de metrô, delegacia, Corpo de Bombeiros, base do SAMU, aeroporto, subestação da Neoenergia.</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr"/>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Faixa fixa</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>&gt; 2.000 m</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>1.500–2.000 m</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>1.000–1.500 m</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>500–1.000 m</t>
+        </is>
+      </c>
+      <c r="K23" s="12" t="inlineStr">
+        <is>
+          <t>≤ 500 m</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>Pedro (03/10/2026)</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>Proposta — conferir se diferencia os 21 pontos</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>CBTU (metrô); Polícia Civil / SDS-PE (delegacias); CBMPE (bombeiros); SAMU; Aeroporto do Recife; Neoenergia (subestações)</t>
+        </is>
+      </c>
+      <c r="O23" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="P23" s="13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="Q23" s="14" t="inlineStr">
+        <is>
+          <t>Lista definida por Pedro. Em aberto: terminais integrados, estruturas da Compesa, Defesa Civil e abrigos. Hospital e UPA ficam no E2. Se quase todos os pontos ficarem acima de 2 km, vira contexto no painel (pendência 18).</t>
+        </is>
+      </c>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>Não pesquisado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Resumo</t>
         </is>
       </c>
-      <c r="O24" s="21" t="inlineStr">
+      <c r="O25" s="21" t="inlineStr">
         <is>
           <t>Fonte confirmada</t>
         </is>
       </c>
-      <c r="P24" s="21" t="inlineStr">
+      <c r="P25" s="21" t="inlineStr">
         <is>
           <t>Dado existe</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="N25" s="22" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="O25" s="23">
-        <f>COUNTIF(O$5:O$22,$N25)</f>
-        <v/>
-      </c>
-      <c r="P25" s="23">
-        <f>COUNTIF(P$5:P$22,$N25)</f>
-        <v/>
       </c>
     </row>
     <row r="26">
       <c r="N26" s="22" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="O26" s="23">
-        <f>COUNTIF(O$5:O$22,$N26)</f>
+        <f>COUNTIF(O$5:O$23,$N26)</f>
         <v/>
       </c>
       <c r="P26" s="23">
-        <f>COUNTIF(P$5:P$22,$N26)</f>
+        <f>COUNTIF(P$5:P$23,$N26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="N27" s="22" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="O27" s="23">
-        <f>COUNTIF(O$5:O$22,$N27)</f>
+        <f>COUNTIF(O$5:O$23,$N27)</f>
         <v/>
       </c>
       <c r="P27" s="23">
-        <f>COUNTIF(P$5:P$22,$N27)</f>
+        <f>COUNTIF(P$5:P$23,$N27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="N28" s="22" t="inlineStr">
         <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="O28" s="23">
+        <f>COUNTIF(O$5:O$23,$N28)</f>
+        <v/>
+      </c>
+      <c r="P28" s="23">
+        <f>COUNTIF(P$5:P$23,$N28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="N29" s="22" t="inlineStr">
+        <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="O28" s="23">
-        <f>COUNTIF(O$5:O$22,$N28)</f>
-        <v/>
-      </c>
-      <c r="P28" s="23">
-        <f>COUNTIF(P$5:P$22,$N28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="N29" s="24" t="inlineStr">
+      <c r="O29" s="23">
+        <f>COUNTIF(O$5:O$23,$N29)</f>
+        <v/>
+      </c>
+      <c r="P29" s="23">
+        <f>COUNTIF(P$5:P$23,$N29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="N30" s="24" t="inlineStr">
         <is>
           <t>Variáveis com fonte e dado confirmados</t>
         </is>
       </c>
-      <c r="P29" s="25">
-        <f>COUNTIFS(O5:O22,"Sim",P5:P22,"Sim")&amp;" de "&amp;ROWS(O5:O22)</f>
+      <c r="P30" s="25">
+        <f>COUNTIFS(O5:O23,"Sim",P5:P23,"Sim")&amp;" de "&amp;ROWS(O5:O23)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:R22"/>
+  <autoFilter ref="A4:R23"/>
   <mergeCells count="1">
     <mergeCell ref="A2:R2"/>
   </mergeCells>
-  <conditionalFormatting sqref="O5:P22">
+  <conditionalFormatting sqref="O5:P23">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Sim"</formula>
     </cfRule>
@@ -2489,7 +2581,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="O5:P22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O5:P23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não,Parcial,Pendente"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
E3: aspecto econômico pela soma do IPTU não residencial em 1 km, notas por quintis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5swnHARNHJ12oc84LP2b9
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
@@ -1607,7 +1607,7 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Nº de comércios e serviços no círculo</t>
+          <t>Soma do IPTU dos imóveis não residenciais no círculo de 1 km (valor lançado; se não houver, o pago). Pontos ordenados e divididos em 5 grupos; empates no mesmo grupo; sem imóvel não residencial = nota 1</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr"/>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>Planilha original</t>
+          <t>Decisão de Pedro (03/10/2026)</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>IBGE — CNEFE 2022 (outras finalidades); IPTU (tipo de empreendimento)</t>
+          <t>Prefeitura do Recife — IPTU 2026 (dados abertos)</t>
         </is>
       </c>
       <c r="O13" s="13" t="inlineStr">
@@ -1668,12 +1668,12 @@
       </c>
       <c r="Q13" s="14" t="inlineStr">
         <is>
-          <t>'Outras finalidades' pode incluir templos e órgãos públicos. Inclui 'perdas econômicas' do documento da equipe, que não tem fonte própria.</t>
+          <t>Aspecto econômico do modelo. Círculo de 1 km (exceção aos 300 m). Isentos entram com valor zero. Nota relativa aos 21 pontos.</t>
         </is>
       </c>
       <c r="R13" s="6" t="inlineStr">
         <is>
-          <t>CNEFE confirmado na busca (não baixado).</t>
+          <t>Segundo Pedro, tem coordenadas e valor pago. Tipo de uso e valor lançado não conferidos.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
E3: fonte de medição IPTU 2026, fonte e dado confirmados por Pedro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5swnHARNHJ12oc84LP2b9
</commit_message>
<xml_diff>
--- a/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
+++ b/dados/Recife_Resiliente_Checklist_Variaveis.xlsx
@@ -1610,7 +1610,11 @@
           <t>Soma do IPTU dos imóveis não residenciais no círculo de 1 km (valor lançado; se não houver, o pago). Pontos ordenados e divididos em 5 grupos; empates no mesmo grupo; sem imóvel não residencial = nota 1</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>IPTU 2026 | Prefeitura do Recife (dados abertos)</t>
+        </is>
+      </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Quintil</t>
@@ -1658,12 +1662,12 @@
       </c>
       <c r="O13" s="13" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="P13" s="13" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="Q13" s="14" t="inlineStr">

</xml_diff>